<commit_message>
Rewrite the data processing pipeline and simplified the visualisation bit
</commit_message>
<xml_diff>
--- a/Data Sources.xlsx
+++ b/Data Sources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/jjw15_ic_ac_uk/Documents/Documents/Grants/25.02 European Talent Academy/Jess, Evi, Nik, Ovidiu/ETA 2025 - Health, biodiversity, food, water nexus/Horizon Europe Connect Fund/Kick-off meeting/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oserban/work/imperial/data-deserts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{10163A94-6627-484E-A9CE-2D398014E33C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463D3461-84B6-6344-A738-5AFB017F06B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="6315" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -453,7 +453,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -478,12 +478,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -499,20 +511,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -536,9 +555,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -576,7 +595,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -682,7 +701,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -824,7 +843,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -853,23 +872,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N19"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="42.42578125" customWidth="1"/>
-    <col min="2" max="2" width="33.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="17.5703125" customWidth="1"/>
-    <col min="9" max="9" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.5703125" customWidth="1"/>
-    <col min="12" max="12" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.5" customWidth="1"/>
+    <col min="2" max="2" width="33.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="17.5" customWidth="1"/>
+    <col min="9" max="9" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.5" customWidth="1"/>
+    <col min="12" max="12" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="33.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -910,211 +929,211 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
-      <c r="A2" t="s">
+    <row r="2" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5">
         <v>2025</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
-      <c r="A3" t="s">
+    <row r="3" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="5">
         <v>2020</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
-      <c r="A4" t="s">
+    <row r="4" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="5">
         <v>2022</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
-      <c r="A5" t="s">
+    <row r="5" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="5">
         <v>2026</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2" t="s">
+      <c r="L5" s="6"/>
+      <c r="M5" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
-      <c r="A6" t="s">
+    <row r="6" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2" t="s">
+      <c r="L6" s="9"/>
+      <c r="M6" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
-      <c r="A7" t="s">
+    <row r="7" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="8">
         <v>2025</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2" t="s">
+      <c r="L7" s="9"/>
+      <c r="M7" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="42.75">
+    <row r="8" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -1137,11 +1156,11 @@
         <v>2025</v>
       </c>
       <c r="L8" s="2"/>
-      <c r="M8" s="5" t="s">
+      <c r="M8" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -1176,115 +1195,115 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="99.75">
-      <c r="A10" t="s">
+    <row r="10" spans="1:14" s="5" customFormat="1" ht="112" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="J10" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="K10" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="L10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="85.5">
-      <c r="A11" t="s">
+    <row r="11" spans="1:14" s="5" customFormat="1" ht="96" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="J11" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="K11" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="M11" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:14" s="3" customFormat="1" ht="42.75">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:14" s="7" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="J12" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="K12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="M12" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N12" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>88</v>
       </c>
@@ -1319,7 +1338,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>95</v>
       </c>
@@ -1348,7 +1367,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>99</v>
       </c>
@@ -1377,7 +1396,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>103</v>
       </c>
@@ -1412,7 +1431,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>106</v>
       </c>
@@ -1444,7 +1463,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>112</v>
       </c>
@@ -1463,7 +1482,7 @@
       <c r="G18" t="s">
         <v>114</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="3">
         <v>46125</v>
       </c>
       <c r="I18" t="s">
@@ -1479,7 +1498,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>118</v>
       </c>
@@ -1528,8 +1547,9 @@
     <hyperlink ref="M19" r:id="rId13" location="dataDownload/Home" xr:uid="{BDEF4F93-4733-47AE-B156-4D0BF37CCF16}"/>
     <hyperlink ref="M7" r:id="rId14" display="https://www.bto.org/get-involved/volunteer/projects/bbs" xr:uid="{DCA522B8-6824-4B0E-BABE-D3387EF02046}"/>
     <hyperlink ref="M11" r:id="rId15" xr:uid="{54BEFAFD-E809-419E-8EAC-3807687E811E}"/>
+    <hyperlink ref="M12" r:id="rId16" xr:uid="{A6F163A5-936F-7646-8738-96BAD654B4C9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId16"/>
+  <legacyDrawing r:id="rId17"/>
 </worksheet>
 </file>
</xml_diff>